<commit_message>
changehistory: add dispositions, categories, and breaking-changes callout for FMG
</commit_message>
<xml_diff>
--- a/output/StructureDefinition-pdex-member-match-group.xlsx
+++ b/output/StructureDefinition-pdex-member-match-group.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1857" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1857" uniqueCount="371">
   <si>
     <t>Property</t>
   </si>
@@ -63,7 +63,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-31T21:00:10-04:00</t>
+    <t>2026-05-29T12:37:47-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -419,7 +419,7 @@
     <t>These resources do not have an independent existence apart from the resource that contains them - they cannot be identified independently, and nor can they have their own independent transaction scope.</t>
   </si>
   <si>
-    <t>Each contained Patient resource SHALL be the exact Patient resource as submitted by the requester in the MemberBundle input parameter, preserving the original resource id, all identifiers, and all demographics supplied by the requester. Responders SHALL NOT abridge or modify the submitted Patient resource. Where the same patient was submitted with multiple different Coverage plans, a contained Coverage resource MAY also be included to identify which (patient + coverage) pair this member entry corresponds to.</t>
+    <t>Each contained Patient resource SHALL be the Patient resource submitted by the requester in the MemberBundle input parameter, preserving the original resource id, all identifier elements, and all demographic elements (name, birthDate, gender, address, telecom, communication, and other Patient elements supplied by the requester) so that the requester can unambiguously correlate each match result back to the submitted member. Responders SHALL NOT modify, abridge, or substitute the submitted Patient resource's id, identifiers, or demographic elements. Per FHIR R4 References (http://hl7.org/fhir/R4/references.html#contained), contained resources SHALL NOT carry meta.versionId, meta.lastUpdated, or meta.security and SHALL NOT themselves contain nested contained resources; where the submitted Patient resource carries any of those base-FHIR-prohibited elements, the responder SHALL remove them when copying the resource into Group.contained[], and doing so is not considered a violation of the preservation requirement. Where the same patient was submitted with multiple different Coverage plans, a contained Coverage resource MAY also be included to identify which (patient + coverage) pair this member entry corresponds to.</t>
   </si>
   <si>
     <t>DomainResource.contained</t>
@@ -521,10 +521,10 @@
     <t>Group.type</t>
   </si>
   <si>
-    <t>person | animal | practitioner | device | medication | substance</t>
-  </si>
-  <si>
-    <t>Identifies the broad classification of the kind of resources the group includes.</t>
+    <t>Type of group (members)</t>
+  </si>
+  <si>
+    <t>Fixed to 'person'. Group.member entries reference Patient resources representing matched members.</t>
   </si>
   <si>
     <t>Group members SHALL be of the appropriate resource type (Patient for person or animal; or Practitioner, Device, Medication or Substance for the other types.).</t>
@@ -533,6 +533,9 @@
     <t>Identifies what type of resources the group is made up of.</t>
   </si>
   <si>
+    <t>person</t>
+  </si>
+  <si>
     <t>required</t>
   </si>
   <si>
@@ -551,10 +554,10 @@
     <t>Group.actual</t>
   </si>
   <si>
-    <t>Descriptive or actual</t>
-  </si>
-  <si>
-    <t>If true, indicates that the resource refers to a specific group of real individuals.  If false, the group defines a set of intended individuals.</t>
+    <t>Actual group (not definitional)</t>
+  </si>
+  <si>
+    <t>An actual list of matched members, not a conceptual/definitional group.</t>
   </si>
   <si>
     <t>There are use-cases for groups that define specific collections of individuals, and other groups that define "types" of intended individuals.  The requirements for both kinds of groups are similar, so we use a single resource, distinguished by this flag.</t>
@@ -636,14 +639,14 @@
     <t>Group.managingEntity</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Organization|4.0.1|RelatedPerson|4.0.1|Practitioner|4.0.1|PractitionerRole|4.0.1)
+    <t xml:space="preserve">Reference(Organization)
 </t>
   </si>
   <si>
-    <t>Entity that is the custodian of the Group's definition</t>
-  </si>
-  <si>
-    <t>Entity responsible for defining and maintaining Group characteristics and/or registered members.</t>
+    <t>Payer managing this group</t>
+  </si>
+  <si>
+    <t>Reference to the Payer organization that created and is managing this matched-member Group. Constrained to Organization since the managing entity is always a Payer (i.e., a healthcare organization), not a Practitioner, PractitionerRole, or RelatedPerson.</t>
   </si>
   <si>
     <t>This does not strictly align with ownership of a herd or flock, but may suffice to represent that relationship in simple cases. More complex cases will require an extension.</t>
@@ -2849,7 +2852,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="13" hidden="true">
+    <row r="13">
       <c r="A13" t="s" s="2">
         <v>161</v>
       </c>
@@ -2868,7 +2871,7 @@
         <v>89</v>
       </c>
       <c r="H13" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="I13" t="s" s="2">
         <v>79</v>
@@ -2899,7 +2902,7 @@
         <v>79</v>
       </c>
       <c r="S13" t="s" s="2">
-        <v>79</v>
+        <v>166</v>
       </c>
       <c r="T13" t="s" s="2">
         <v>79</v>
@@ -2914,13 +2917,13 @@
         <v>79</v>
       </c>
       <c r="X13" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="Y13" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="Z13" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="AA13" t="s" s="2">
         <v>79</v>
@@ -2953,18 +2956,18 @@
         <v>101</v>
       </c>
       <c r="AK13" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="14" hidden="true">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="14">
       <c r="A14" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2978,7 +2981,7 @@
         <v>89</v>
       </c>
       <c r="H14" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="I14" t="s" s="2">
         <v>79</v>
@@ -2990,14 +2993,14 @@
         <v>154</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" t="s" s="2">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P14" t="s" s="2">
         <v>79</v>
@@ -3007,7 +3010,7 @@
         <v>79</v>
       </c>
       <c r="S14" t="s" s="2">
-        <v>79</v>
+        <v>13</v>
       </c>
       <c r="T14" t="s" s="2">
         <v>79</v>
@@ -3046,7 +3049,7 @@
         <v>79</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>89</v>
@@ -3055,24 +3058,24 @@
         <v>89</v>
       </c>
       <c r="AI14" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AJ14" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AK14" t="s" s="2">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AL14" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -3095,16 +3098,16 @@
         <v>90</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="N15" t="s" s="2">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="O15" s="2"/>
       <c r="P15" t="s" s="2">
@@ -3130,11 +3133,11 @@
         <v>79</v>
       </c>
       <c r="X15" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="Y15" s="2"/>
       <c r="Z15" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AA15" t="s" s="2">
         <v>79</v>
@@ -3152,7 +3155,7 @@
         <v>79</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>80</v>
@@ -3167,18 +3170,18 @@
         <v>101</v>
       </c>
       <c r="AK15" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AL15" t="s" s="2">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -3201,17 +3204,17 @@
         <v>90</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" t="s" s="2">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="P16" t="s" s="2">
         <v>79</v>
@@ -3260,7 +3263,7 @@
         <v>79</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>80</v>
@@ -3275,7 +3278,7 @@
         <v>101</v>
       </c>
       <c r="AK16" t="s" s="2">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="AL16" t="s" s="2">
         <v>79</v>
@@ -3283,10 +3286,10 @@
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3309,19 +3312,19 @@
         <v>90</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="N17" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="O17" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="P17" t="s" s="2">
         <v>79</v>
@@ -3370,7 +3373,7 @@
         <v>79</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>80</v>
@@ -3385,7 +3388,7 @@
         <v>101</v>
       </c>
       <c r="AK17" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="AL17" t="s" s="2">
         <v>79</v>
@@ -3393,10 +3396,10 @@
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -3419,16 +3422,16 @@
         <v>90</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="N18" t="s" s="2">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -3478,7 +3481,7 @@
         <v>79</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>80</v>
@@ -3501,10 +3504,10 @@
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3527,19 +3530,19 @@
         <v>79</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="O19" t="s" s="2">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="P19" t="s" s="2">
         <v>79</v>
@@ -3588,7 +3591,7 @@
         <v>79</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>80</v>
@@ -3603,7 +3606,7 @@
         <v>101</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="AL19" t="s" s="2">
         <v>79</v>
@@ -3611,10 +3614,10 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -3637,13 +3640,13 @@
         <v>79</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -3694,7 +3697,7 @@
         <v>79</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>80</v>
@@ -3709,7 +3712,7 @@
         <v>79</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AL20" t="s" s="2">
         <v>79</v>
@@ -3717,10 +3720,10 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3749,7 +3752,7 @@
         <v>136</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="N21" t="s" s="2">
         <v>138</v>
@@ -3802,7 +3805,7 @@
         <v>79</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>80</v>
@@ -3817,7 +3820,7 @@
         <v>140</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AL21" t="s" s="2">
         <v>79</v>
@@ -3825,14 +3828,14 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s" s="2">
@@ -3854,10 +3857,10 @@
         <v>135</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="N22" t="s" s="2">
         <v>138</v>
@@ -3912,7 +3915,7 @@
         <v>79</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>80</v>
@@ -3935,10 +3938,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3961,17 +3964,17 @@
         <v>79</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="P23" t="s" s="2">
         <v>79</v>
@@ -3996,10 +3999,10 @@
         <v>79</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="Y23" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="Z23" t="s" s="2">
         <v>79</v>
@@ -4020,7 +4023,7 @@
         <v>79</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>89</v>
@@ -4035,7 +4038,7 @@
         <v>101</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AL23" t="s" s="2">
         <v>79</v>
@@ -4043,10 +4046,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4069,13 +4072,13 @@
         <v>79</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -4126,7 +4129,7 @@
         <v>79</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>80</v>
@@ -4141,7 +4144,7 @@
         <v>79</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AL24" t="s" s="2">
         <v>79</v>
@@ -4149,10 +4152,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4181,7 +4184,7 @@
         <v>136</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="N25" t="s" s="2">
         <v>138</v>
@@ -4222,19 +4225,19 @@
         <v>79</v>
       </c>
       <c r="AB25" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="AC25" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AD25" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE25" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>80</v>
@@ -4249,7 +4252,7 @@
         <v>140</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AL25" t="s" s="2">
         <v>79</v>
@@ -4257,10 +4260,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4283,19 +4286,19 @@
         <v>90</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="O26" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>79</v>
@@ -4320,11 +4323,11 @@
         <v>79</v>
       </c>
       <c r="X26" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="Y26" s="2"/>
       <c r="Z26" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="AA26" t="s" s="2">
         <v>79</v>
@@ -4342,7 +4345,7 @@
         <v>79</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>80</v>
@@ -4357,7 +4360,7 @@
         <v>101</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AL26" t="s" s="2">
         <v>79</v>
@@ -4365,10 +4368,10 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4391,13 +4394,13 @@
         <v>79</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -4448,7 +4451,7 @@
         <v>79</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>80</v>
@@ -4463,7 +4466,7 @@
         <v>79</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AL27" t="s" s="2">
         <v>79</v>
@@ -4471,10 +4474,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4503,7 +4506,7 @@
         <v>136</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="N28" t="s" s="2">
         <v>138</v>
@@ -4544,19 +4547,19 @@
         <v>79</v>
       </c>
       <c r="AB28" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="AC28" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AD28" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE28" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>80</v>
@@ -4571,7 +4574,7 @@
         <v>140</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AL28" t="s" s="2">
         <v>79</v>
@@ -4579,10 +4582,10 @@
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4608,16 +4611,16 @@
         <v>103</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="O29" t="s" s="2">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>79</v>
@@ -4666,7 +4669,7 @@
         <v>79</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>80</v>
@@ -4681,7 +4684,7 @@
         <v>101</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="AL29" t="s" s="2">
         <v>79</v>
@@ -4689,10 +4692,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4715,16 +4718,16 @@
         <v>90</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
@@ -4774,7 +4777,7 @@
         <v>79</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>80</v>
@@ -4789,7 +4792,7 @@
         <v>101</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AL30" t="s" s="2">
         <v>79</v>
@@ -4797,10 +4800,10 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4826,14 +4829,14 @@
         <v>109</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="P31" t="s" s="2">
         <v>79</v>
@@ -4843,7 +4846,7 @@
         <v>79</v>
       </c>
       <c r="S31" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="T31" t="s" s="2">
         <v>79</v>
@@ -4882,7 +4885,7 @@
         <v>79</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>80</v>
@@ -4897,7 +4900,7 @@
         <v>101</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="AL31" t="s" s="2">
         <v>79</v>
@@ -4905,10 +4908,10 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -4931,17 +4934,17 @@
         <v>90</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P32" t="s" s="2">
         <v>79</v>
@@ -4990,7 +4993,7 @@
         <v>79</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>80</v>
@@ -5005,7 +5008,7 @@
         <v>101</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="AL32" t="s" s="2">
         <v>79</v>
@@ -5013,10 +5016,10 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5042,16 +5045,16 @@
         <v>154</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="O33" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="P33" t="s" s="2">
         <v>79</v>
@@ -5100,7 +5103,7 @@
         <v>79</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>80</v>
@@ -5115,7 +5118,7 @@
         <v>101</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="AL33" t="s" s="2">
         <v>79</v>
@@ -5123,10 +5126,10 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5149,19 +5152,19 @@
         <v>90</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="O34" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>79</v>
@@ -5210,7 +5213,7 @@
         <v>79</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>80</v>
@@ -5225,7 +5228,7 @@
         <v>101</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="AL34" t="s" s="2">
         <v>79</v>
@@ -5233,10 +5236,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5259,19 +5262,19 @@
         <v>79</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="O35" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="P35" t="s" s="2">
         <v>79</v>
@@ -5296,10 +5299,10 @@
         <v>79</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="Y35" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="Z35" t="s" s="2">
         <v>79</v>
@@ -5308,17 +5311,17 @@
         <v>79</v>
       </c>
       <c r="AB35" t="s" s="2">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="AC35" s="2"/>
       <c r="AD35" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE35" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>89</v>
@@ -5333,7 +5336,7 @@
         <v>101</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="AL35" t="s" s="2">
         <v>79</v>
@@ -5341,13 +5344,13 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C36" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D36" t="s" s="2">
         <v>79</v>
@@ -5369,19 +5372,19 @@
         <v>79</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="O36" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>79</v>
@@ -5430,7 +5433,7 @@
         <v>79</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>89</v>
@@ -5445,7 +5448,7 @@
         <v>101</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>79</v>
@@ -5453,10 +5456,10 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5482,16 +5485,16 @@
         <v>154</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="O37" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="P37" t="s" s="2">
         <v>79</v>
@@ -5540,7 +5543,7 @@
         <v>79</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>89</v>
@@ -5555,7 +5558,7 @@
         <v>101</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>79</v>
@@ -5563,10 +5566,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5589,16 +5592,16 @@
         <v>79</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="N38" t="s" s="2">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
@@ -5648,7 +5651,7 @@
         <v>79</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>80</v>
@@ -5671,10 +5674,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5697,17 +5700,17 @@
         <v>79</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="P39" t="s" s="2">
         <v>79</v>
@@ -5756,7 +5759,7 @@
         <v>79</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>80</v>
@@ -5765,13 +5768,13 @@
         <v>81</v>
       </c>
       <c r="AI39" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AJ39" t="s" s="2">
         <v>101</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="AL39" t="s" s="2">
         <v>79</v>
@@ -5779,10 +5782,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5805,13 +5808,13 @@
         <v>79</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -5862,7 +5865,7 @@
         <v>79</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>80</v>
@@ -5877,7 +5880,7 @@
         <v>79</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AL40" t="s" s="2">
         <v>79</v>
@@ -5885,10 +5888,10 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -5917,7 +5920,7 @@
         <v>136</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="N41" t="s" s="2">
         <v>138</v>
@@ -5970,7 +5973,7 @@
         <v>79</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>80</v>
@@ -5985,7 +5988,7 @@
         <v>140</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AL41" t="s" s="2">
         <v>79</v>
@@ -5993,14 +5996,14 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
@@ -6022,10 +6025,10 @@
         <v>135</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="N42" t="s" s="2">
         <v>138</v>
@@ -6080,7 +6083,7 @@
         <v>79</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>80</v>
@@ -6103,10 +6106,10 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6129,13 +6132,13 @@
         <v>79</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -6186,7 +6189,7 @@
         <v>79</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>89</v>
@@ -6209,10 +6212,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6235,13 +6238,13 @@
         <v>79</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
@@ -6292,7 +6295,7 @@
         <v>79</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>80</v>
@@ -6307,7 +6310,7 @@
         <v>79</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AL44" t="s" s="2">
         <v>79</v>
@@ -6315,10 +6318,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6344,10 +6347,10 @@
         <v>135</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -6386,19 +6389,19 @@
         <v>79</v>
       </c>
       <c r="AB45" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="AC45" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="AD45" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE45" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>80</v>
@@ -6421,13 +6424,13 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C46" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D46" t="s" s="2">
         <v>79</v>
@@ -6449,16 +6452,16 @@
         <v>79</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="N46" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
@@ -6508,7 +6511,7 @@
         <v>79</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>80</v>
@@ -6531,13 +6534,13 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C47" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D47" t="s" s="2">
         <v>79</v>
@@ -6559,16 +6562,16 @@
         <v>79</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="N47" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -6618,7 +6621,7 @@
         <v>79</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>80</v>
@@ -6641,10 +6644,10 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -6667,16 +6670,16 @@
         <v>90</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="N48" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O48" s="2"/>
       <c r="P48" t="s" s="2">
@@ -6726,7 +6729,7 @@
         <v>79</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>80</v>
@@ -6735,7 +6738,7 @@
         <v>89</v>
       </c>
       <c r="AI48" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="AJ48" t="s" s="2">
         <v>101</v>
@@ -6749,10 +6752,10 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -6778,13 +6781,13 @@
         <v>103</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="N49" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
@@ -6810,13 +6813,13 @@
         <v>79</v>
       </c>
       <c r="X49" t="s" s="2">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="Y49" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="Z49" t="s" s="2">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="AA49" t="s" s="2">
         <v>79</v>
@@ -6834,7 +6837,7 @@
         <v>79</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>80</v>
@@ -6857,10 +6860,10 @@
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -6886,13 +6889,13 @@
         <v>147</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="N50" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="O50" s="2"/>
       <c r="P50" t="s" s="2">
@@ -6942,7 +6945,7 @@
         <v>79</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>80</v>
@@ -6957,7 +6960,7 @@
         <v>101</v>
       </c>
       <c r="AK50" t="s" s="2">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="AL50" t="s" s="2">
         <v>79</v>
@@ -6965,10 +6968,10 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -6991,16 +6994,16 @@
         <v>90</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="N51" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="O51" s="2"/>
       <c r="P51" t="s" s="2">
@@ -7050,7 +7053,7 @@
         <v>79</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>80</v>
@@ -7073,10 +7076,10 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -7099,23 +7102,23 @@
         <v>79</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="N52" s="2"/>
       <c r="O52" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="P52" t="s" s="2">
         <v>79</v>
       </c>
       <c r="Q52" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="R52" t="s" s="2">
         <v>79</v>
@@ -7160,7 +7163,7 @@
         <v>79</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>80</v>
@@ -7183,10 +7186,10 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7212,20 +7215,20 @@
         <v>154</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="P53" t="s" s="2">
         <v>79</v>
       </c>
       <c r="Q53" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="R53" t="s" s="2">
         <v>79</v>
@@ -7270,7 +7273,7 @@
         <v>79</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>80</v>

</xml_diff>